<commit_message>
Added a model option to specify the sheet in the people excel so the hospital people behaviour can be varied. Added different behaviour sheets to the workbook, and a bulk scenario to compare them.
</commit_message>
<xml_diff>
--- a/InputData/people.xlsx
+++ b/InputData/people.xlsx
@@ -5,13 +5,17 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="people_details" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="default" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="no_common" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="dept_only" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">people_details!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">default!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">dept_only!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">no_common!$1:$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="27">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -34,73 +38,13 @@
     <t xml:space="preserve">AREA: large animal</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">AREA: </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Small animal</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">AREA: </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Farm services</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">AREA: </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">common</t>
-    </r>
+    <t xml:space="preserve">AREA: Small animal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREA: Farm services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREA: common</t>
   </si>
   <si>
     <t xml:space="preserve">ADI</t>
@@ -173,7 +117,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -210,13 +154,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -261,7 +198,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -276,10 +213,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -322,13 +255,13 @@
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="AMD1" s="1"/>
@@ -616,6 +549,608 @@
         <v>10</v>
       </c>
     </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.2" right="0.7" top="0.5" bottom="0.5" header="0.3" footer="0.511811023622047"/>
+  <pageSetup paperSize="5" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;L&amp;"Calibri,Bold Italic"&amp;8Updated Apr 1/22&amp;C&amp;"Arial,Bold"&amp;14ACTIVE HEALTH MANAGEMENT CLIENTS</oddHeader>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:AMJ13"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.32"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="8" style="1" width="9.14"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="2" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AMD1" s="1"/>
+      <c r="AME1" s="1"/>
+      <c r="AMF1" s="1"/>
+      <c r="AMG1" s="1"/>
+      <c r="AMH1" s="1"/>
+      <c r="AMI1" s="1"/>
+      <c r="AMJ1" s="0"/>
+    </row>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" s="2" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AMD12" s="1"/>
+      <c r="AME12" s="1"/>
+      <c r="AMF12" s="1"/>
+      <c r="AMG12" s="1"/>
+      <c r="AMH12" s="1"/>
+      <c r="AMI12" s="1"/>
+      <c r="AMJ12" s="0"/>
+    </row>
+    <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.2" right="0.7" top="0.5" bottom="0.5" header="0.3" footer="0.511811023622047"/>
+  <pageSetup paperSize="5" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;L&amp;"Calibri,Bold Italic"&amp;8Updated Apr 1/22&amp;C&amp;"Arial,Bold"&amp;14ACTIVE HEALTH MANAGEMENT CLIENTS</oddHeader>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:AMJ1048576"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="17.35" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.32"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="8" style="1" width="9.14"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="2" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AMD1" s="1"/>
+      <c r="AME1" s="1"/>
+      <c r="AMF1" s="1"/>
+      <c r="AMG1" s="1"/>
+      <c r="AMH1" s="1"/>
+      <c r="AMI1" s="1"/>
+      <c r="AMJ1" s="0"/>
+    </row>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.2" right="0.7" top="0.5" bottom="0.5" header="0.3" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
- fixed cleaning schedules - works for scenarios in 260206 paper version     - Quarantine -> truck clean -> vaccination
</commit_message>
<xml_diff>
--- a/InputData/people.xlsx
+++ b/InputData/people.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" state="visible" r:id="rId2"/>
@@ -44,7 +44,7 @@
     <t xml:space="preserve">AREA: Farm services</t>
   </si>
   <si>
-    <t xml:space="preserve">AREA: common</t>
+    <t xml:space="preserve">AREA: common area</t>
   </si>
   <si>
     <t xml:space="preserve">ADI</t>
@@ -907,7 +907,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.39"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="8" style="1" width="9.14"/>
   </cols>
   <sheetData>

</xml_diff>